<commit_message>
new big ticket items
</commit_message>
<xml_diff>
--- a/Africa Important Dates.xlsx
+++ b/Africa Important Dates.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\JN1PEPF00000647\EXCELCNV\559e54c3-e4c4-418d-9bb4-782d7e60a9d4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3DB5EAD9-6623-4F4D-AC32-B3EC31151281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{3DB5EAD9-6623-4F4D-AC32-B3EC31151281}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{70F574DD-3CE3-4025-B3CA-062B1F1C2F24}"/>
   <bookViews>
     <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Big Ticket Activities" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Important Dates'!$A$1:$G$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Important Dates'!$A$1:$G$103</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="768" uniqueCount="215">
   <si>
     <t>Country</t>
   </si>
@@ -276,421 +276,412 @@
     <t>Dealer Activation - Linex: Pretoria Airshow</t>
   </si>
   <si>
+    <t>04-Sep-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation: Linex: 24HR MTB Race Activation</t>
+  </si>
+  <si>
+    <t>Tanzania</t>
+  </si>
+  <si>
+    <t>12-Sep-2026</t>
+  </si>
+  <si>
+    <t>Customer Experience Project - 125 5G, Morogoro</t>
+  </si>
+  <si>
+    <t>HLX Day</t>
+  </si>
+  <si>
+    <t>Customer appreciation. Fun family day with HLX riders</t>
+  </si>
+  <si>
+    <t>Customer Engagement</t>
+  </si>
+  <si>
     <t>Kenya</t>
   </si>
   <si>
-    <t>04-Sep-2026</t>
+    <t>14-Sep-2026</t>
+  </si>
+  <si>
+    <t>Africa on Apache</t>
+  </si>
+  <si>
+    <t>Ghana</t>
+  </si>
+  <si>
+    <t>15-Sep-2026</t>
+  </si>
+  <si>
+    <t>HLX DAY</t>
+  </si>
+  <si>
+    <t>Nigeria</t>
+  </si>
+  <si>
+    <t>HLX Day Community Day</t>
+  </si>
+  <si>
+    <t>18-Sep-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation - TWK Activation</t>
+  </si>
+  <si>
+    <t>19-Sep-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation - Linex: Scooter Run</t>
+  </si>
+  <si>
+    <t>21-Sep-2026</t>
+  </si>
+  <si>
+    <t>Apache RTR 180 Mall Activation</t>
+  </si>
+  <si>
+    <t>Africa on Apache Campaign</t>
+  </si>
+  <si>
+    <t>26-Sep-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation - Tex Motorcycles:  Outeniqua Family Market</t>
+  </si>
+  <si>
+    <t>27-Sep-2026</t>
+  </si>
+  <si>
+    <t>Concours de Elegance</t>
+  </si>
+  <si>
+    <t>28-Sep-2026</t>
+  </si>
+  <si>
+    <t>3S Inaugartion at Diego</t>
+  </si>
+  <si>
+    <t>30-Sep-2026</t>
+  </si>
+  <si>
+    <t>3S Inaugartion at Fort Dhauphin &amp; Assembly area opening</t>
+  </si>
+  <si>
+    <t>03-Oct-2026</t>
+  </si>
+  <si>
+    <t>HLX Day Dar</t>
+  </si>
+  <si>
+    <t>10-Oct-2026</t>
+  </si>
+  <si>
+    <t>HLX Day Mwanza</t>
+  </si>
+  <si>
+    <t>Senegal</t>
+  </si>
+  <si>
+    <t>15-Oct-2026</t>
+  </si>
+  <si>
+    <t>AOG Ride</t>
+  </si>
+  <si>
+    <t>First AOG Ride</t>
+  </si>
+  <si>
+    <t>16-Oct-2026</t>
+  </si>
+  <si>
+    <t>Tanzania Bikers Festival</t>
+  </si>
+  <si>
+    <t>17-Oct-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation - Linex Demo Day</t>
+  </si>
+  <si>
+    <t>20-Oct-2026</t>
+  </si>
+  <si>
+    <t>HLX &amp; NEO BTL Campaign (Roadshow &amp; Test Ride)</t>
+  </si>
+  <si>
+    <t>BTL Campaign</t>
+  </si>
+  <si>
+    <t>Marketing Activity</t>
+  </si>
+  <si>
+    <t>Neo Day</t>
+  </si>
+  <si>
+    <t>Neo Day Community Building</t>
+  </si>
+  <si>
+    <t>Liberia</t>
+  </si>
+  <si>
+    <t>22-Oct-2026</t>
+  </si>
+  <si>
+    <t>Apache 180 Refresh Soft Launch</t>
+  </si>
+  <si>
+    <t>Launch of Apache in the market</t>
+  </si>
+  <si>
+    <t>Jupiter Launch Event</t>
+  </si>
+  <si>
+    <t>Ronin Launch with media from the store</t>
+  </si>
+  <si>
+    <t>23-Oct-2026</t>
+  </si>
+  <si>
+    <t>Boda Festival - Arusha</t>
+  </si>
+  <si>
+    <t>25-Oct-2026</t>
+  </si>
+  <si>
+    <t>HLX Family Day Community Building</t>
+  </si>
+  <si>
+    <t>Bikers Lives Matter</t>
+  </si>
+  <si>
+    <t>28-Oct-2026</t>
+  </si>
+  <si>
+    <t>3W Queen Ride Project</t>
+  </si>
+  <si>
+    <t>01-Nov-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation - Bay City Auto Killarney Motor Show</t>
+  </si>
+  <si>
+    <t>06-Nov-2026</t>
+  </si>
+  <si>
+    <t>Dealer Activation - Tex Motorcycles: Kwagga Golf Day</t>
+  </si>
+  <si>
+    <t>Sierra Leone</t>
+  </si>
+  <si>
+    <t>10-Nov-2026</t>
+  </si>
+  <si>
+    <t>IQube Launch</t>
+  </si>
+  <si>
+    <t>Launch of IQUBE 1st EV in West Africa</t>
+  </si>
+  <si>
+    <t>TBC</t>
+  </si>
+  <si>
+    <t>KZN Mass Recruitment</t>
+  </si>
+  <si>
+    <t>Pretoria mass recruitment</t>
+  </si>
+  <si>
+    <t>September</t>
+  </si>
+  <si>
+    <t>3W GS+ Seeding Units</t>
+  </si>
+  <si>
+    <t>Customer Experience Project - 125 5G, Arusha</t>
+  </si>
+  <si>
+    <t>October</t>
+  </si>
+  <si>
+    <t>Customer Experience Project - 125 5G, Dodoma</t>
+  </si>
+  <si>
+    <t>Customer Experience Project - 125 5G, Iringa</t>
+  </si>
+  <si>
+    <t>Customer Experience Project - 125 5G, Musoma</t>
+  </si>
+  <si>
+    <t>Customer Experience Project - Plus, Tanga</t>
+  </si>
+  <si>
+    <t>Demovan Lake Zone</t>
+  </si>
+  <si>
+    <t>Demovan South Zone</t>
+  </si>
+  <si>
+    <t>November</t>
+  </si>
+  <si>
+    <t>HLX Day (1 Dar, 1 Mbeya)</t>
+  </si>
+  <si>
+    <t>ITrust HLX Rally</t>
+  </si>
+  <si>
+    <t>Load Test Campaign</t>
+  </si>
+  <si>
+    <t>Mega Mileage Test Ride</t>
+  </si>
+  <si>
+    <t>Mega Service Camp (Dar - 3 Nos), Lake - 2 Nos</t>
+  </si>
+  <si>
+    <t>Mega Service Camp (Dar - 3 Nos), South - 2 Nos, North -1</t>
+  </si>
+  <si>
+    <t>Mega Service Camp 5 Nos</t>
+  </si>
+  <si>
+    <t>Mini FSC (6 Nos)</t>
+  </si>
+  <si>
+    <t>Mini FSC (8 Nos)</t>
+  </si>
+  <si>
+    <t>Minor Mileage Test Ride</t>
+  </si>
+  <si>
+    <t>New Coco 2S inauguration - Matwara</t>
+  </si>
+  <si>
+    <t>New Coco 2S inauguration - Tanga</t>
+  </si>
+  <si>
+    <t>Own Demovan Central</t>
+  </si>
+  <si>
+    <t>Own Demovan Coastal</t>
+  </si>
+  <si>
+    <t>Own Demovan Dar</t>
+  </si>
+  <si>
+    <t>Own Demovan Pwani</t>
+  </si>
+  <si>
+    <t>Radio Campaign (Arusha, Mbeya, Dodoma, Mwanza, Dar, Morogoro, Iringa, Kahama, Moshi, Tanga, Singida,)</t>
+  </si>
+  <si>
+    <t>Trial Bike HLX 125 5G, Kahama</t>
+  </si>
+  <si>
+    <t>Armado Launch</t>
+  </si>
+  <si>
+    <t>iQube Launch</t>
+  </si>
+  <si>
+    <t>Guinea</t>
+  </si>
+  <si>
+    <t>Apache 180 Refresh Launch</t>
+  </si>
+  <si>
+    <t>Ivory Coast</t>
+  </si>
+  <si>
+    <t>Apache 180 Refresh Launch, Neo Dual tone Launch &amp; Korhogo Branch Inauguration </t>
+  </si>
+  <si>
+    <t>EV (IQUBE, ORBITER &amp; KING EV Maxx launch)</t>
+  </si>
+  <si>
+    <t>Cameroon</t>
+  </si>
+  <si>
+    <t>2nd Distributor Appointment, Showroom Launch &amp; PR Amplification</t>
+  </si>
+  <si>
+    <t>HLX 100 CC AGD - Nyanza</t>
+  </si>
+  <si>
+    <t>HLX 100 CC AGD - Coast</t>
+  </si>
+  <si>
+    <t>HLX 100 CC AGD - Rift / Western</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>AOG Kickoff</t>
+  </si>
+  <si>
+    <t>ARE</t>
+  </si>
+  <si>
+    <t>Tunisia</t>
+  </si>
+  <si>
+    <t>Market Entry</t>
+  </si>
+  <si>
+    <t>Mauritania</t>
+  </si>
+  <si>
+    <t>Angola</t>
+  </si>
+  <si>
+    <t>Ethiopia</t>
+  </si>
+  <si>
+    <t>EV Portfolio Launch</t>
+  </si>
+  <si>
+    <t>Malawi</t>
+  </si>
+  <si>
+    <t>Zambia</t>
+  </si>
+  <si>
+    <t>DRC</t>
+  </si>
+  <si>
+    <t>Jupiter &amp; Ronin Launch</t>
+  </si>
+  <si>
+    <t>Mauritius</t>
+  </si>
+  <si>
+    <t>RTR 310 Launch</t>
+  </si>
+  <si>
+    <t>SOW vehicle Launch -10 Units</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antenna Dealer meet </t>
+  </si>
+  <si>
+    <t>Nyeri Polytechnic College  - PTC Center</t>
   </si>
   <si>
     <t>Meru Store Opening</t>
   </si>
   <si>
-    <t>Postponed</t>
-  </si>
-  <si>
-    <t>Dealer Activation: Linex: 24HR MTB Race Activation</t>
-  </si>
-  <si>
-    <t>Tanzania</t>
-  </si>
-  <si>
-    <t>12-Sep-2026</t>
-  </si>
-  <si>
-    <t>Customer Experience Project - 125 5G, Morogoro</t>
-  </si>
-  <si>
-    <t>HLX Day</t>
-  </si>
-  <si>
-    <t>Customer appreciation. Fun family day with HLX riders</t>
-  </si>
-  <si>
-    <t>Customer Engagement</t>
-  </si>
-  <si>
-    <t>14-Sep-2026</t>
-  </si>
-  <si>
-    <t>Africa on Apache</t>
-  </si>
-  <si>
-    <t>Ghana</t>
-  </si>
-  <si>
-    <t>15-Sep-2026</t>
-  </si>
-  <si>
-    <t>HLX DAY</t>
-  </si>
-  <si>
-    <t>Nigeria</t>
-  </si>
-  <si>
-    <t>HLX Day Community Day</t>
-  </si>
-  <si>
-    <t>18-Sep-2026</t>
-  </si>
-  <si>
-    <t>Dealer Activation - TWK Activation</t>
-  </si>
-  <si>
-    <t>19-Sep-2026</t>
-  </si>
-  <si>
-    <t>Dealer Activation - Linex: Scooter Run</t>
-  </si>
-  <si>
-    <t>21-Sep-2026</t>
-  </si>
-  <si>
-    <t>Apache RTR 180 Mall Activation</t>
-  </si>
-  <si>
-    <t>Africa on Apache Campaign</t>
-  </si>
-  <si>
-    <t>26-Sep-2026</t>
-  </si>
-  <si>
-    <t>Dealer Activation - Tex Motorcycles:  Outeniqua Family Market</t>
-  </si>
-  <si>
-    <t>27-Sep-2026</t>
-  </si>
-  <si>
-    <t>Concours de Elegance</t>
-  </si>
-  <si>
-    <t>28-Sep-2026</t>
-  </si>
-  <si>
-    <t>3S Inaugartion at Diego</t>
-  </si>
-  <si>
-    <t>30-Sep-2026</t>
-  </si>
-  <si>
-    <t>3S Inaugartion at Fort Dhauphin &amp; Assembly area opening</t>
-  </si>
-  <si>
-    <t>03-Oct-2026</t>
-  </si>
-  <si>
-    <t>HLX Day Dar</t>
-  </si>
-  <si>
-    <t>10-Oct-2026</t>
-  </si>
-  <si>
-    <t>HLX Day Mwanza</t>
-  </si>
-  <si>
-    <t>Senegal</t>
-  </si>
-  <si>
-    <t>15-Oct-2026</t>
-  </si>
-  <si>
-    <t>AOG Ride</t>
-  </si>
-  <si>
-    <t>First AOG Ride</t>
-  </si>
-  <si>
-    <t>16-Oct-2026</t>
-  </si>
-  <si>
-    <t>Tanzania Bikers Festival</t>
-  </si>
-  <si>
-    <t>17-Oct-2026</t>
-  </si>
-  <si>
-    <t>Dealer Activation - Linex Demo Day</t>
-  </si>
-  <si>
-    <t>20-Oct-2026</t>
-  </si>
-  <si>
-    <t>HLX &amp; NEO BTL Campaign (Roadshow &amp; Test Ride)</t>
-  </si>
-  <si>
-    <t>BTL Campaign</t>
-  </si>
-  <si>
-    <t>Marketing Activity</t>
-  </si>
-  <si>
-    <t>Neo Day</t>
-  </si>
-  <si>
-    <t>Neo Day Community Building</t>
-  </si>
-  <si>
-    <t>Liberia</t>
-  </si>
-  <si>
-    <t>22-Oct-2026</t>
-  </si>
-  <si>
-    <t>Apache 180 Refresh Soft Launch</t>
-  </si>
-  <si>
-    <t>Launch of Apache in the market</t>
-  </si>
-  <si>
-    <t>Jupiter Launch Event</t>
-  </si>
-  <si>
-    <t>Ronin Launch with media from the store</t>
-  </si>
-  <si>
-    <t>23-Oct-2026</t>
-  </si>
-  <si>
-    <t>Boda Festival - Arusha</t>
-  </si>
-  <si>
-    <t>Guinea</t>
-  </si>
-  <si>
-    <t>25-Oct-2026</t>
-  </si>
-  <si>
     <t>Apache rtr 180 Launch</t>
   </si>
   <si>
-    <t>HLX Family Day Community Building</t>
-  </si>
-  <si>
-    <t>Bikers Lives Matter</t>
-  </si>
-  <si>
-    <t>28-Oct-2026</t>
-  </si>
-  <si>
-    <t>3W Queen Ride Project</t>
-  </si>
-  <si>
-    <t>01-Nov-2026</t>
-  </si>
-  <si>
-    <t>Dealer Activation - Bay City Auto Killarney Motor Show</t>
-  </si>
-  <si>
-    <t>06-Nov-2026</t>
-  </si>
-  <si>
-    <t>Dealer Activation - Tex Motorcycles: Kwagga Golf Day</t>
-  </si>
-  <si>
-    <t>Sierra Leone</t>
-  </si>
-  <si>
-    <t>10-Nov-2026</t>
-  </si>
-  <si>
-    <t>IQube Launch</t>
-  </si>
-  <si>
-    <t>Launch of IQUBE 1st EV in West Africa</t>
-  </si>
-  <si>
-    <t>20-21 Nov 2026</t>
-  </si>
-  <si>
-    <t>Apache Track day and RTR310 Launch</t>
-  </si>
-  <si>
     <t>27-Nov-2026</t>
   </si>
   <si>
     <t>Raider I-Go, NTORQ 150 Launch</t>
-  </si>
-  <si>
-    <t>TBC</t>
-  </si>
-  <si>
-    <t>KZN Mass Recruitment</t>
-  </si>
-  <si>
-    <t>Pretoria mass recruitment</t>
-  </si>
-  <si>
-    <t>September</t>
-  </si>
-  <si>
-    <t>3W GS+ Seeding Units</t>
-  </si>
-  <si>
-    <t>Customer Experience Project - 125 5G, Arusha</t>
-  </si>
-  <si>
-    <t>October</t>
-  </si>
-  <si>
-    <t>Customer Experience Project - 125 5G, Dodoma</t>
-  </si>
-  <si>
-    <t>Customer Experience Project - 125 5G, Iringa</t>
-  </si>
-  <si>
-    <t>Customer Experience Project - 125 5G, Musoma</t>
-  </si>
-  <si>
-    <t>Customer Experience Project - Plus, Tanga</t>
-  </si>
-  <si>
-    <t>Demovan Lake Zone</t>
-  </si>
-  <si>
-    <t>Demovan South Zone</t>
-  </si>
-  <si>
-    <t>November</t>
-  </si>
-  <si>
-    <t>HLX Day (1 Dar, 1 Mbeya)</t>
-  </si>
-  <si>
-    <t>ITrust HLX Rally</t>
-  </si>
-  <si>
-    <t>Load Test Campaign</t>
-  </si>
-  <si>
-    <t>Mega Mileage Test Ride</t>
-  </si>
-  <si>
-    <t>Mega Service Camp (Dar - 3 Nos), Lake - 2 Nos</t>
-  </si>
-  <si>
-    <t>Mega Service Camp (Dar - 3 Nos), South - 2 Nos, North -1</t>
-  </si>
-  <si>
-    <t>Mega Service Camp 5 Nos</t>
-  </si>
-  <si>
-    <t>Mini FSC (6 Nos)</t>
-  </si>
-  <si>
-    <t>Mini FSC (8 Nos)</t>
-  </si>
-  <si>
-    <t>Minor Mileage Test Ride</t>
-  </si>
-  <si>
-    <t>New Coco 2S inauguration - Matwara</t>
-  </si>
-  <si>
-    <t>New Coco 2S inauguration - Tanga</t>
-  </si>
-  <si>
-    <t>Own Demovan Central</t>
-  </si>
-  <si>
-    <t>Own Demovan Coastal</t>
-  </si>
-  <si>
-    <t>Own Demovan Dar</t>
-  </si>
-  <si>
-    <t>Own Demovan Pwani</t>
-  </si>
-  <si>
-    <t>Radio Campaign (Arusha, Mbeya, Dodoma, Mwanza, Dar, Morogoro, Iringa, Kahama, Moshi, Tanga, Singida,)</t>
-  </si>
-  <si>
-    <t>Trial Bike HLX 125 5G, Kahama</t>
-  </si>
-  <si>
-    <t>Armado Launch</t>
-  </si>
-  <si>
-    <t>iQube Launch</t>
-  </si>
-  <si>
-    <t>Apache 180 Refresh Launch</t>
-  </si>
-  <si>
-    <t>Ivory Coast</t>
-  </si>
-  <si>
-    <t>Apache 180 Refresh Launch, Neo Dual tone Launch &amp; Korhogo Branch Inauguration </t>
-  </si>
-  <si>
-    <t>EV (IQUBE, ORBITER &amp; KING EV Maxx launch)</t>
-  </si>
-  <si>
-    <t>Cameroon</t>
-  </si>
-  <si>
-    <t>2nd Distributor Appointment, Showroom Launch &amp; PR Amplification</t>
-  </si>
-  <si>
-    <t>HLX 100 CC AGD - Nyanza</t>
-  </si>
-  <si>
-    <t>HLX 100 CC AGD - Coast</t>
-  </si>
-  <si>
-    <t>HLX 100 CC AGD - Rift / Western</t>
-  </si>
-  <si>
-    <t>Egypt</t>
-  </si>
-  <si>
-    <t>AOG Kickoff</t>
-  </si>
-  <si>
-    <t>ARE</t>
-  </si>
-  <si>
-    <t>Tunisia</t>
-  </si>
-  <si>
-    <t>Market Entry</t>
-  </si>
-  <si>
-    <t>Mauritania</t>
-  </si>
-  <si>
-    <t>Angola</t>
-  </si>
-  <si>
-    <t>Ethiopia</t>
-  </si>
-  <si>
-    <t>EV Portfolio Launch</t>
-  </si>
-  <si>
-    <t>Malawi</t>
-  </si>
-  <si>
-    <t>Zambia</t>
-  </si>
-  <si>
-    <t>DRC</t>
-  </si>
-  <si>
-    <t>Jupiter &amp; Ronin Launch</t>
-  </si>
-  <si>
-    <t>Mauritius</t>
-  </si>
-  <si>
-    <t>RTR 310 Launch</t>
-  </si>
-  <si>
-    <t>SOW vehicle Launch -10 Units</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Antenna Dealer meet </t>
-  </si>
-  <si>
-    <t>Nyeri Polytechnic College  - PTC Center</t>
   </si>
   <si>
     <t> </t>
@@ -1251,7 +1242,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G107"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1829,7 +1820,7 @@
         <v>75</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E26" s="9"/>
       <c r="F26" s="9" t="s">
@@ -1862,16 +1853,16 @@
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="C28" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="9" t="s">
-        <v>80</v>
-      </c>
       <c r="D28" s="7" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="E28" s="9"/>
       <c r="F28" s="9" t="s">
@@ -1881,66 +1872,66 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:7">
+    <row r="29" spans="1:7" ht="30.75">
       <c r="A29" s="9" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>82</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="9" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="30.75">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="C30" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C30" s="9" t="s">
-        <v>85</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E30" s="9"/>
+      <c r="E30" s="9" t="s">
+        <v>84</v>
+      </c>
       <c r="F30" s="9" t="s">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="30.75">
       <c r="A31" s="9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>87</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="E31" s="9"/>
       <c r="F31" s="9" t="s">
-        <v>88</v>
+        <v>28</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>13</v>
@@ -1948,34 +1939,36 @@
     </row>
     <row r="32" spans="1:7" ht="30.75">
       <c r="A32" s="9" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E32" s="9"/>
+      <c r="E32" s="9" t="s">
+        <v>91</v>
+      </c>
       <c r="F32" s="9" t="s">
         <v>28</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="30.75">
       <c r="A33" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>46</v>
@@ -1990,27 +1983,25 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="30.75">
+    <row r="34" spans="1:7">
       <c r="A34" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B34" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="B34" s="9" t="s">
-        <v>92</v>
-      </c>
       <c r="C34" s="9" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E34" s="9" t="s">
-        <v>95</v>
-      </c>
+      <c r="E34" s="9"/>
       <c r="F34" s="9" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -2034,9 +2025,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
+    <row r="36" spans="1:7" ht="30.75">
       <c r="A36" s="9" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="B36" s="9" t="s">
         <v>98</v>
@@ -2049,7 +2040,7 @@
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G36" s="9" t="s">
         <v>13</v>
@@ -2057,13 +2048,13 @@
     </row>
     <row r="37" spans="1:7" ht="30.75">
       <c r="A37" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B37" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>100</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>101</v>
       </c>
       <c r="D37" s="7" t="s">
         <v>46</v>
@@ -2078,10 +2069,10 @@
     </row>
     <row r="38" spans="1:7" ht="30.75">
       <c r="A38" s="9" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>102</v>
@@ -2091,7 +2082,7 @@
       </c>
       <c r="E38" s="9"/>
       <c r="F38" s="9" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>13</v>
@@ -2099,7 +2090,7 @@
     </row>
     <row r="39" spans="1:7" ht="30.75">
       <c r="A39" s="9" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="B39" s="9" t="s">
         <v>103</v>
@@ -2112,15 +2103,15 @@
       </c>
       <c r="E39" s="9"/>
       <c r="F39" s="9" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="30.75">
+    <row r="40" spans="1:7">
       <c r="A40" s="9" t="s">
-        <v>78</v>
+        <v>7</v>
       </c>
       <c r="B40" s="9" t="s">
         <v>105</v>
@@ -2133,7 +2124,7 @@
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>13</v>
@@ -2160,9 +2151,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="1:7">
+    <row r="42" spans="1:7" ht="30.75">
       <c r="A42" s="9" t="s">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="B42" s="9" t="s">
         <v>109</v>
@@ -2175,15 +2166,15 @@
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="30.75">
       <c r="A43" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B43" s="9" t="s">
         <v>111</v>
@@ -2204,18 +2195,20 @@
     </row>
     <row r="44" spans="1:7" ht="30.75">
       <c r="A44" s="9" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C44" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D44" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E44" s="9"/>
+      <c r="E44" s="9" t="s">
+        <v>116</v>
+      </c>
       <c r="F44" s="9" t="s">
         <v>28</v>
       </c>
@@ -2225,30 +2218,28 @@
     </row>
     <row r="45" spans="1:7" ht="30.75">
       <c r="A45" s="9" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D45" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E45" s="9" t="s">
-        <v>118</v>
-      </c>
+      <c r="E45" s="9"/>
       <c r="F45" s="9" t="s">
         <v>28</v>
       </c>
       <c r="G45" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="30.75">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" s="9" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>119</v>
@@ -2261,7 +2252,7 @@
       </c>
       <c r="E46" s="9"/>
       <c r="F46" s="9" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>13</v>
@@ -2269,7 +2260,7 @@
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="9" t="s">
-        <v>14</v>
+        <v>89</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>121</v>
@@ -2280,66 +2271,68 @@
       <c r="D47" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E47" s="9"/>
+      <c r="E47" s="9" t="s">
+        <v>123</v>
+      </c>
       <c r="F47" s="9" t="s">
-        <v>20</v>
+        <v>124</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="30.75">
       <c r="A48" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D48" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>126</v>
+        <v>28</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="30.75">
+    <row r="49" spans="1:7">
       <c r="A49" s="9" t="s">
-        <v>94</v>
+        <v>127</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" s="9" t="s">
-        <v>129</v>
+        <v>7</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>131</v>
@@ -2347,9 +2340,7 @@
       <c r="D50" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E50" s="9" t="s">
-        <v>132</v>
-      </c>
+      <c r="E50" s="9"/>
       <c r="F50" s="9" t="s">
         <v>12</v>
       </c>
@@ -2362,10 +2353,10 @@
         <v>7</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D51" s="7" t="s">
         <v>46</v>
@@ -2378,12 +2369,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
+    <row r="52" spans="1:7" ht="30.75">
       <c r="A52" s="9" t="s">
-        <v>7</v>
+        <v>80</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C52" s="9" t="s">
         <v>134</v>
@@ -2393,26 +2384,28 @@
       </c>
       <c r="E52" s="9"/>
       <c r="F52" s="9" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="30.75">
       <c r="A53" s="9" t="s">
-        <v>83</v>
+        <v>113</v>
       </c>
       <c r="B53" s="9" t="s">
         <v>135</v>
       </c>
       <c r="C53" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E53" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="D53" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E53" s="9"/>
       <c r="F53" s="9" t="s">
         <v>28</v>
       </c>
@@ -2420,58 +2413,54 @@
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:7" ht="30.75">
       <c r="A54" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="C54" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B54" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>139</v>
-      </c>
       <c r="D54" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E54" s="9" t="s">
-        <v>132</v>
-      </c>
+      <c r="E54" s="9"/>
       <c r="F54" s="9" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="30.75">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" s="9" t="s">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="B55" s="9" t="s">
         <v>138</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>86</v>
+        <v>139</v>
       </c>
       <c r="D55" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E55" s="9" t="s">
-        <v>140</v>
-      </c>
+      <c r="E55" s="9"/>
       <c r="F55" s="9" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="30.75">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" s="9" t="s">
         <v>14</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C56" s="9" t="s">
         <v>141</v>
@@ -2481,15 +2470,15 @@
       </c>
       <c r="E56" s="9"/>
       <c r="F56" s="9" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" s="9" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="B57" s="9" t="s">
         <v>142</v>
@@ -2502,7 +2491,7 @@
       </c>
       <c r="E57" s="9"/>
       <c r="F57" s="9" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>13</v>
@@ -2510,52 +2499,54 @@
     </row>
     <row r="58" spans="1:7">
       <c r="A58" s="9" t="s">
-        <v>14</v>
+        <v>144</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C58" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D58" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E58" s="9"/>
+      <c r="E58" s="9" t="s">
+        <v>147</v>
+      </c>
       <c r="F58" s="9" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:7" ht="30.75">
       <c r="A59" s="9" t="s">
         <v>14</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D59" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E59" s="9"/>
       <c r="F59" s="9" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="30.75">
       <c r="A60" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B60" s="9" t="s">
         <v>148</v>
-      </c>
-      <c r="B60" s="9" t="s">
-        <v>149</v>
       </c>
       <c r="C60" s="9" t="s">
         <v>150</v>
@@ -2563,67 +2554,65 @@
       <c r="D60" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E60" s="9" t="s">
+      <c r="E60" s="9"/>
+      <c r="F60" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="30.75">
+      <c r="A61" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B61" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="F60" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="G60" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
-      <c r="A61" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B61" s="9" t="s">
+      <c r="C61" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C61" s="9" t="s">
-        <v>153</v>
-      </c>
       <c r="D61" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E61" s="9"/>
       <c r="F61" s="9" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="30.75">
       <c r="A62" s="9" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E62" s="9"/>
       <c r="F62" s="9" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="30.75">
       <c r="A63" s="9" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D63" s="7" t="s">
         <v>46</v>
@@ -2638,16 +2627,16 @@
     </row>
     <row r="64" spans="1:7" ht="30.75">
       <c r="A64" s="9" t="s">
-        <v>14</v>
+        <v>80</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C64" s="9" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E64" s="9"/>
       <c r="F64" s="9" t="s">
@@ -2659,16 +2648,16 @@
     </row>
     <row r="65" spans="1:7" ht="30.75">
       <c r="A65" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C65" s="9" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="E65" s="9"/>
       <c r="F65" s="9" t="s">
@@ -2680,16 +2669,16 @@
     </row>
     <row r="66" spans="1:7" ht="30.75">
       <c r="A66" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C66" s="9" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="E66" s="9"/>
       <c r="F66" s="9" t="s">
@@ -2701,13 +2690,13 @@
     </row>
     <row r="67" spans="1:7" ht="30.75">
       <c r="A67" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="D67" s="7" t="s">
         <v>46</v>
@@ -2722,16 +2711,16 @@
     </row>
     <row r="68" spans="1:7" ht="30.75">
       <c r="A68" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B68" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C68" s="9" t="s">
-        <v>163</v>
+        <v>82</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="E68" s="9"/>
       <c r="F68" s="9" t="s">
@@ -2743,16 +2732,16 @@
     </row>
     <row r="69" spans="1:7" ht="30.75">
       <c r="A69" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E69" s="9"/>
       <c r="F69" s="9" t="s">
@@ -2764,13 +2753,13 @@
     </row>
     <row r="70" spans="1:7" ht="30.75">
       <c r="A70" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C70" s="9" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="D70" s="7" t="s">
         <v>46</v>
@@ -2785,13 +2774,13 @@
     </row>
     <row r="71" spans="1:7" ht="30.75">
       <c r="A71" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D71" s="7" t="s">
         <v>46</v>
@@ -2804,57 +2793,57 @@
         <v>29</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="30.75">
+    <row r="72" spans="1:7">
       <c r="A72" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B72" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C72" s="9" t="s">
-        <v>85</v>
+        <v>159</v>
       </c>
       <c r="D72" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E72" s="9"/>
       <c r="F72" s="9" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="30.75">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7">
       <c r="A73" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="E73" s="9"/>
       <c r="F73" s="9" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="30.75">
       <c r="A74" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B74" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C74" s="9" t="s">
         <v>162</v>
-      </c>
-      <c r="C74" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="D74" s="7" t="s">
         <v>46</v>
@@ -2869,13 +2858,13 @@
     </row>
     <row r="75" spans="1:7" ht="30.75">
       <c r="A75" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B75" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C75" s="9" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D75" s="7" t="s">
         <v>46</v>
@@ -2888,106 +2877,106 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:7">
+    <row r="76" spans="1:7" ht="30.75">
       <c r="A76" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B76" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C76" s="9" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D76" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E76" s="9"/>
       <c r="F76" s="9" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B77" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D77" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E77" s="9"/>
       <c r="F77" s="9" t="s">
-        <v>65</v>
+        <v>124</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" ht="30.75">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
       <c r="A78" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="C78" s="9" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="D78" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E78" s="9"/>
       <c r="F78" s="9" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="G78" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="30.75">
+    <row r="79" spans="1:7">
       <c r="A79" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B79" s="9" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C79" s="9" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D79" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E79" s="9"/>
       <c r="F79" s="9" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="G79" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="80" spans="1:7" ht="30.75">
+    <row r="80" spans="1:7">
       <c r="A80" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C80" s="9" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D80" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E80" s="9"/>
       <c r="F80" s="9" t="s">
-        <v>28</v>
+        <v>124</v>
       </c>
       <c r="G80" s="9" t="s">
         <v>29</v>
@@ -2995,83 +2984,83 @@
     </row>
     <row r="81" spans="1:7">
       <c r="A81" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B81" s="9" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C81" s="9" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D81" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E81" s="9"/>
       <c r="F81" s="9" t="s">
-        <v>126</v>
+        <v>65</v>
       </c>
       <c r="G81" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B82" s="9" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C82" s="9" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="D82" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E82" s="9"/>
       <c r="F82" s="9" t="s">
-        <v>126</v>
+        <v>65</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C83" s="9" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="D83" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E83" s="9"/>
       <c r="F83" s="9" t="s">
-        <v>126</v>
+        <v>65</v>
       </c>
       <c r="G83" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D84" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E84" s="9"/>
       <c r="F84" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G84" s="9" t="s">
         <v>29</v>
@@ -3079,83 +3068,83 @@
     </row>
     <row r="85" spans="1:7">
       <c r="A85" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C85" s="9" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="D85" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E85" s="9"/>
       <c r="F85" s="9" t="s">
-        <v>65</v>
+        <v>124</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="86" spans="1:7">
       <c r="A86" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C86" s="9" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="D86" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E86" s="9"/>
       <c r="F86" s="9" t="s">
-        <v>65</v>
+        <v>124</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="87" spans="1:7">
       <c r="A87" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B87" s="9" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="C87" s="9" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="D87" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E87" s="9"/>
       <c r="F87" s="9" t="s">
-        <v>65</v>
+        <v>124</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
     </row>
     <row r="88" spans="1:7">
       <c r="A88" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B88" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C88" s="9" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D88" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E88" s="9"/>
       <c r="F88" s="9" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G88" s="9" t="s">
         <v>29</v>
@@ -3163,104 +3152,104 @@
     </row>
     <row r="89" spans="1:7">
       <c r="A89" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B89" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C89" s="9" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D89" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E89" s="9"/>
       <c r="F89" s="9" t="s">
-        <v>126</v>
+        <v>20</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="90" spans="1:7">
       <c r="A90" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B90" s="9" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C90" s="9" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="D90" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E90" s="9"/>
       <c r="F90" s="9" t="s">
-        <v>126</v>
+        <v>20</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="91" spans="1:7">
       <c r="A91" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B91" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C91" s="9" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="D91" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E91" s="9"/>
       <c r="F91" s="9" t="s">
-        <v>126</v>
+        <v>65</v>
       </c>
       <c r="G91" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="92" spans="1:7">
       <c r="A92" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C92" s="9" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D92" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E92" s="9"/>
       <c r="F92" s="9" t="s">
-        <v>126</v>
+        <v>65</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="93" spans="1:7">
       <c r="A93" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B93" s="9" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="C93" s="9" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D93" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E93" s="9"/>
       <c r="F93" s="9" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="G93" s="9" t="s">
         <v>13</v>
@@ -3268,192 +3257,144 @@
     </row>
     <row r="94" spans="1:7">
       <c r="A94" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B94" s="9" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
       <c r="C94" s="9" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D94" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E94" s="9"/>
       <c r="F94" s="9" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="G94" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
+    <row r="95" spans="1:7" ht="30.75">
       <c r="A95" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C95" s="9" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D95" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E95" s="9"/>
       <c r="F95" s="9" t="s">
-        <v>65</v>
+        <v>124</v>
       </c>
       <c r="G95" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" ht="30.75">
       <c r="A96" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B96" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C96" s="9" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="D96" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E96" s="9"/>
       <c r="F96" s="9" t="s">
-        <v>65</v>
+        <v>124</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="30.75">
       <c r="A97" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B97" s="9" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="C97" s="9" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D97" s="7" t="s">
-        <v>46</v>
+        <v>10</v>
       </c>
       <c r="E97" s="9"/>
       <c r="F97" s="9" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="G97" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="30.75">
       <c r="A98" s="9" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C98" s="9" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="D98" s="7" t="s">
         <v>46</v>
       </c>
       <c r="E98" s="9"/>
       <c r="F98" s="9" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" ht="30.75">
-      <c r="A99" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B99" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="C99" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="D99" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E99" s="9"/>
-      <c r="F99" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="G99" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" ht="30.75">
-      <c r="A100" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B100" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="C100" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="D100" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E100" s="9"/>
-      <c r="F100" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="G100" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" ht="30.75">
-      <c r="A101" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="C101" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="D101" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E101" s="9"/>
-      <c r="F101" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="G101" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" ht="30.75">
-      <c r="A102" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B102" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="C102" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="D102" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="E102" s="9"/>
-      <c r="F102" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="G102" s="9" t="s">
-        <v>29</v>
-      </c>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7">
+      <c r="A99" s="1"/>
+      <c r="B99" s="1"/>
+      <c r="C99" s="1"/>
+      <c r="D99" s="1"/>
+      <c r="E99" s="1"/>
+      <c r="F99" s="1"/>
+      <c r="G99" s="1"/>
+    </row>
+    <row r="100" spans="1:7">
+      <c r="A100" s="1"/>
+      <c r="B100" s="1"/>
+      <c r="C100" s="1"/>
+      <c r="D100" s="1"/>
+      <c r="E100" s="1"/>
+      <c r="F100" s="1"/>
+      <c r="G100" s="1"/>
+    </row>
+    <row r="101" spans="1:7">
+      <c r="A101" s="1"/>
+      <c r="B101" s="1"/>
+      <c r="C101" s="1"/>
+      <c r="D101" s="1"/>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1"/>
+      <c r="G101" s="1"/>
+    </row>
+    <row r="102" spans="1:7">
+      <c r="A102" s="1"/>
+      <c r="B102" s="1"/>
+      <c r="C102" s="1"/>
+      <c r="D102" s="1"/>
+      <c r="E102" s="1"/>
+      <c r="F102" s="1"/>
+      <c r="G102" s="1"/>
     </row>
     <row r="103" spans="1:7">
       <c r="A103" s="1"/>
@@ -3464,45 +3405,9 @@
       <c r="F103" s="1"/>
       <c r="G103" s="1"/>
     </row>
-    <row r="104" spans="1:7">
-      <c r="A104" s="1"/>
-      <c r="B104" s="1"/>
-      <c r="C104" s="1"/>
-      <c r="D104" s="1"/>
-      <c r="E104" s="1"/>
-      <c r="F104" s="1"/>
-      <c r="G104" s="1"/>
-    </row>
-    <row r="105" spans="1:7">
-      <c r="A105" s="1"/>
-      <c r="B105" s="1"/>
-      <c r="C105" s="1"/>
-      <c r="D105" s="1"/>
-      <c r="E105" s="1"/>
-      <c r="F105" s="1"/>
-      <c r="G105" s="1"/>
-    </row>
-    <row r="106" spans="1:7">
-      <c r="A106" s="1"/>
-      <c r="B106" s="1"/>
-      <c r="C106" s="1"/>
-      <c r="D106" s="1"/>
-      <c r="E106" s="1"/>
-      <c r="F106" s="1"/>
-      <c r="G106" s="1"/>
-    </row>
-    <row r="107" spans="1:7">
-      <c r="A107" s="1"/>
-      <c r="B107" s="1"/>
-      <c r="C107" s="1"/>
-      <c r="D107" s="1"/>
-      <c r="E107" s="1"/>
-      <c r="F107" s="1"/>
-      <c r="G107" s="1"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G107" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="D78:D102 D15:D21">
+  <autoFilter ref="A1:G103" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="D74:D98 D15:D21 D27:D28 D31:D60">
     <cfRule type="cellIs" dxfId="20" priority="19" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
@@ -3513,7 +3418,7 @@
       <formula>"Executed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D14 D22:D24 D32:D64 D67 D69:D72 D74:D77 D27:D29">
+  <conditionalFormatting sqref="D14 D22:D24 D63 D65:D68 D70:D73">
     <cfRule type="cellIs" dxfId="17" priority="13" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
@@ -3535,7 +3440,7 @@
       <formula>"Executed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D65:D66 D68 D73 D30:D31">
+  <conditionalFormatting sqref="D61:D62 D64 D69 D29:D30">
     <cfRule type="cellIs" dxfId="11" priority="7" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
@@ -3569,7 +3474,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D102" xr:uid="{B73B4048-65AC-4180-B5CE-9FC78A3C8476}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D98" xr:uid="{B73B4048-65AC-4180-B5CE-9FC78A3C8476}">
       <formula1>"Executed, Postponed, Yet to Happen"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3616,13 +3521,13 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B2" s="6">
         <v>46351</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>46</v>
@@ -3637,13 +3542,13 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B3" s="6">
         <v>46336</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>46</v>
@@ -3658,13 +3563,13 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="4" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="B4" s="6">
         <v>46346</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>46</v>
@@ -3679,13 +3584,13 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B5" s="6">
         <v>46351</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>46</v>
@@ -3700,13 +3605,13 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="B6" s="6">
         <v>46315</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>46</v>
@@ -3721,13 +3626,13 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B7" s="6">
         <v>46341</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>46</v>
@@ -3742,13 +3647,13 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B8" s="6">
         <v>46320</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>46</v>
@@ -3763,13 +3668,13 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B9" s="6">
         <v>46334</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>46</v>
@@ -3784,13 +3689,13 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B10" s="6">
         <v>46340</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>46</v>
@@ -3805,13 +3710,13 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B11" s="6">
         <v>46342</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>46</v>
@@ -3826,13 +3731,13 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="4" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B12" s="6">
         <v>46305</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>46</v>
@@ -3847,13 +3752,13 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="4" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B13" s="6">
         <v>46336</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>46</v>
@@ -3868,13 +3773,13 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="4" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B14" s="6">
         <v>46351</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>46</v>
@@ -3889,13 +3794,13 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="4" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B15" s="6">
         <v>46362</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>46</v>
@@ -3910,13 +3815,13 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="4" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="B16" s="6">
         <v>46322</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>46</v>
@@ -3931,13 +3836,13 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="4" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B17" s="6">
         <v>46344</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>46</v>
@@ -3952,13 +3857,13 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="4" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="B18" s="6">
         <v>46338</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>46</v>
@@ -3973,13 +3878,13 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="4" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="B19" s="6">
         <v>46347</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>46</v>
@@ -3994,13 +3899,13 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="4" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B20" s="6">
         <v>46350</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>46</v>
@@ -4021,7 +3926,7 @@
         <v>46317</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>46</v>
@@ -4036,13 +3941,13 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="4" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="B22" s="6">
         <v>46329</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>46</v>
@@ -4063,7 +3968,7 @@
         <v>46342</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="D23" s="7" t="s">
         <v>46</v>
@@ -4078,13 +3983,13 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B24" s="6">
         <v>46323</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D24" s="7" t="s">
         <v>46</v>
@@ -4099,13 +4004,13 @@
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="8" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B25" s="6">
         <v>46294</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>46</v>
@@ -4120,13 +4025,13 @@
     </row>
     <row r="26" spans="1:7">
       <c r="A26" s="8" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B26" s="6">
         <v>46321</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>46</v>
@@ -4141,13 +4046,13 @@
     </row>
     <row r="27" spans="1:7">
       <c r="A27" s="8" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="B27" s="6">
         <v>46323</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>46</v>
@@ -4160,9 +4065,70 @@
         <v>13</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="15.75">
-      <c r="F30" s="2"/>
-      <c r="G30" s="3"/>
+    <row r="28" spans="1:7">
+      <c r="A28" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="6">
+        <v>46290</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="31" spans="1:7" ht="15.75">
       <c r="F31" s="2"/>
@@ -4174,23 +4140,23 @@
     </row>
     <row r="33" spans="6:6" ht="15.75">
       <c r="F33" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D1:E1 D2:D27">
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+  <conditionalFormatting sqref="D1:E1 D2:D30">
+    <cfRule type="cellIs" dxfId="2" priority="10" operator="equal">
       <formula>"Yet to Happen"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="11" operator="equal">
       <formula>"Postponed"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="12" operator="equal">
       <formula>"Executed"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D27" xr:uid="{5E8D2655-5D3D-4C03-89C3-96D784A677A4}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D30" xr:uid="{5E8D2655-5D3D-4C03-89C3-96D784A677A4}">
       <formula1>"Executed, Postponed, Yet to Happen"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F27" xr:uid="{5EF1DAAA-68F2-4547-91DA-5A249D40B114}">

</xml_diff>